<commit_message>
Fix duplicate email issue - make email unique per run
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/UserRegistrationData.xlsx
+++ b/src/test/resources/testdata/UserRegistrationData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{A22A524C-3CDF-47D9-A513-F7E72F5F18D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{744C58FA-AEE0-41F7-B4DE-8E87416FBE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,28 +73,28 @@
     <t>WrongPass@123</t>
   </si>
   <si>
-    <t>pushpa</t>
-  </si>
-  <si>
-    <t>allu</t>
-  </si>
-  <si>
-    <t>bahu</t>
-  </si>
-  <si>
-    <t>bali</t>
-  </si>
-  <si>
-    <t>pushpa.allu1944@testmail.com</t>
-  </si>
-  <si>
-    <t>bahu.bali79@testmail.com</t>
-  </si>
-  <si>
-    <t>Test@1289</t>
-  </si>
-  <si>
-    <t>Test@8956</t>
+    <t>hit</t>
+  </si>
+  <si>
+    <t>man</t>
+  </si>
+  <si>
+    <t>king</t>
+  </si>
+  <si>
+    <t>kohli</t>
+  </si>
+  <si>
+    <t>hit.man84@testmail.com</t>
+  </si>
+  <si>
+    <t>king.kohli63@testmail.com</t>
+  </si>
+  <si>
+    <t>Test@12897</t>
+  </si>
+  <si>
+    <t>Test@89564</t>
   </si>
 </sst>
 </file>
@@ -523,7 +523,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="2">
-        <v>9876538210</v>
+        <v>9876534510</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -552,7 +552,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="2">
-        <v>9184456780</v>
+        <v>9184456718</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Update test data in xlsx
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/UserRegistrationData.xlsx
+++ b/src/test/resources/testdata/UserRegistrationData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{744C58FA-AEE0-41F7-B4DE-8E87416FBE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{109CF7A0-8070-463C-828D-85C1C7159168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,28 +73,28 @@
     <t>WrongPass@123</t>
   </si>
   <si>
-    <t>hit</t>
-  </si>
-  <si>
-    <t>man</t>
-  </si>
-  <si>
-    <t>king</t>
-  </si>
-  <si>
-    <t>kohli</t>
-  </si>
-  <si>
-    <t>hit.man84@testmail.com</t>
-  </si>
-  <si>
-    <t>king.kohli63@testmail.com</t>
-  </si>
-  <si>
-    <t>Test@12897</t>
-  </si>
-  <si>
-    <t>Test@89564</t>
+    <t>shiva</t>
+  </si>
+  <si>
+    <t>lord</t>
+  </si>
+  <si>
+    <t>shiva.lord65@testmail.com</t>
+  </si>
+  <si>
+    <t>namo</t>
+  </si>
+  <si>
+    <t>om</t>
+  </si>
+  <si>
+    <t>namo.om78@testmail.com</t>
+  </si>
+  <si>
+    <t>Test@1297</t>
+  </si>
+  <si>
+    <t>Test@8964</t>
   </si>
 </sst>
 </file>
@@ -520,10 +520,10 @@
         <v>19</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2">
-        <v>9876534510</v>
+        <v>9812534510</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -543,16 +543,16 @@
         <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E3" s="2">
-        <v>9184456718</v>
+        <v>9167456718</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Fix User2 LastName - must be 3+ characters
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/UserRegistrationData.xlsx
+++ b/src/test/resources/testdata/UserRegistrationData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{109CF7A0-8070-463C-828D-85C1C7159168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5ED07311-F4E8-47FC-95B7-84B2A81EF5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,28 +73,28 @@
     <t>WrongPass@123</t>
   </si>
   <si>
-    <t>shiva</t>
-  </si>
-  <si>
     <t>lord</t>
   </si>
   <si>
-    <t>shiva.lord65@testmail.com</t>
-  </si>
-  <si>
     <t>namo</t>
   </si>
   <si>
-    <t>om</t>
-  </si>
-  <si>
-    <t>namo.om78@testmail.com</t>
-  </si>
-  <si>
     <t>Test@1297</t>
   </si>
   <si>
     <t>Test@8964</t>
+  </si>
+  <si>
+    <t>shivay</t>
+  </si>
+  <si>
+    <t>venkatesaya</t>
+  </si>
+  <si>
+    <t>shivay.lord65@testmail.com</t>
+  </si>
+  <si>
+    <t>namo.venkatesaya78@testmail.com</t>
   </si>
 </sst>
 </file>
@@ -514,16 +514,16 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="D2" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2">
-        <v>9812534510</v>
+        <v>9812534512</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -532,10 +532,10 @@
         <v>11</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -543,16 +543,16 @@
         <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E3" s="2">
-        <v>9167456718</v>
+        <v>9167456719</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>13</v>
@@ -561,10 +561,10 @@
         <v>14</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>